<commit_message>
feat!: ship Blend Kit 2.0 with report 2.4 and automation testing
Keep one report format and the existing Test Spec source readers. Support
reviewed evidence writeback for RC-001 source 1.1 without changing its source.

Remove legacy assets, migration code, archives and obsolete build snapshots.
Use one canonical runtime, current JA/VI templates and explicit image slots.
Update workflow documentation, packaging and regression coverage.
</commit_message>
<xml_diff>
--- a/dist/plugins/blend-kit/skills/blend-generate-task/_kit/skills/blend-generate-test-spec/assets/test-report-block-template.ja.xlsx
+++ b/dist/plugins/blend-kit/skills/blend-generate-task/_kit/skills/blend-generate-test-spec/assets/test-report-block-template.ja.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:workbook xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <ns0:workbookPr filterPrivacy="1"/>
-  <ns0:bookViews>
-    <ns0:workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-2025" windowWidth="29040" windowHeight="17520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </ns0:bookViews>
-  <ns0:sheets>
-    <ns0:sheet name="概要" sheetId="1" state="visible" ns1:id="rId1"/>
-    <ns0:sheet name="テストケース" sheetId="2" state="visible" ns1:id="rId2"/>
-  </ns0:sheets>
-  <ns0:definedNames>
-    <ns0:definedName name="_xlnm.Print_Area" localSheetId="1">'テストケース'!$A$1:$E$21</ns0:definedName>
-  </ns0:definedNames>
-  <ns0:calcPr calcId="181029" fullCalcOnLoad="1"/>
-</ns0:workbook>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-2025" windowWidth="29040" windowHeight="17520" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet name="概要" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="テストケース" sheetId="2" state="visible" r:id="rId2"/>
+  </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'概要'!$A$29:$C$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'概要'!$A$1:$C$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'テストケース'!$A$1:$F$93</definedName>
+  </definedNames>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
+</workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -21,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -81,6 +83,23 @@
       <b val="1"/>
       <color rgb="00172033"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <color rgb="00172033"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <color rgb="001D4ED8"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <b val="1"/>
+      <color rgb="00172033"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="9">
@@ -126,7 +145,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -148,11 +167,109 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <bottom style="thin">
+        <color rgb="00D9E2EC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9E2EC"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9E2EC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E2EC"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9E2EC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E2EC"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9E2EC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E2EC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E2EC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9E2EC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9E2EC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E2EC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E2EC"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9E2EC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9E2EC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E2EC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9E2EC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E2EC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9E2EC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E2EC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E2EC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -274,6 +391,93 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="8" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="8" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="8" borderId="7" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -549,9 +753,9 @@
   <sheetPr>
     <tabColor rgb="00334155"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -568,7 +772,7 @@
       <c r="B1" s="10" t="n"/>
     </row>
     <row r="2" ht="12" customHeight="1">
-      <c r="A2" s="10" t="n"/>
+      <c r="A2" s="10" t="inlineStr"/>
       <c r="B2" s="10" t="n"/>
     </row>
     <row r="3" ht="32.1" customHeight="1">
@@ -578,98 +782,119 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="32.1" customHeight="1">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="27" t="inlineStr">
         <is>
           <t>機能</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n"/>
-    </row>
-    <row r="5" ht="32.1" customHeight="1">
+      <c r="B4" s="49" t="inlineStr">
+        <is>
+          <t>SYN-SC synthetic rule lifecycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
           <t>テスト設計版</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n"/>
-    </row>
-    <row r="6" ht="32.1" customHeight="1">
+      <c r="B5" s="49" t="inlineStr">
+        <is>
+          <t>compact-r1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="27" t="inlineStr">
         <is>
           <t>テスト実行ID</t>
         </is>
       </c>
-      <c r="B6" s="28" t="n"/>
-      <c r="C6" s="29" t="n"/>
-    </row>
-    <row r="7" ht="32.1" customHeight="1">
+      <c r="B6" s="50" t="inlineStr"/>
+      <c r="C6" s="64" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="27" t="inlineStr">
         <is>
           <t>アプリケーション版</t>
         </is>
       </c>
-      <c r="B7" s="28" t="n"/>
-      <c r="C7" s="29" t="n"/>
-    </row>
-    <row r="8" ht="32.1" customHeight="1">
+      <c r="B7" s="50" t="inlineStr"/>
+      <c r="C7" s="64" t="n"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="27" t="inlineStr">
         <is>
           <t>環境</t>
         </is>
       </c>
-      <c r="B8" s="28" t="n"/>
-      <c r="C8" s="29" t="n"/>
-    </row>
-    <row r="9" ht="32.1" customHeight="1">
+      <c r="B8" s="50" t="inlineStr"/>
+      <c r="C8" s="64" t="n"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="27" t="inlineStr">
         <is>
           <t>実施者</t>
         </is>
       </c>
-      <c r="B9" s="28" t="n"/>
-      <c r="C9" s="29" t="n"/>
-    </row>
-    <row r="10" ht="32.1" customHeight="1">
+      <c r="B9" s="50" t="inlineStr"/>
+      <c r="C9" s="64" t="n"/>
+    </row>
+    <row r="10" ht="44" customHeight="1">
       <c r="A10" s="27" t="inlineStr">
         <is>
           <t>実施日時（タイムゾーン付き）</t>
         </is>
       </c>
-      <c r="B10" s="28" t="n"/>
-      <c r="C10" s="29" t="n"/>
-    </row>
-    <row r="11" ht="32.1" customHeight="1">
+      <c r="B10" s="50" t="inlineStr"/>
+      <c r="C10" s="64" t="n"/>
+    </row>
+    <row r="11" ht="78" customHeight="1">
       <c r="A11" s="27" t="inlineStr">
         <is>
           <t>対象範囲</t>
         </is>
       </c>
-      <c r="B11" s="10" t="n"/>
-    </row>
-    <row r="12" ht="32.1" customHeight="1">
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>SYN:O1–O8; boundary, deletion, incomplete/stale rule, AND controls
+準備: TD-SC create/verify/reset once per variant; G-PREP retains unknown entry/readback seams
+開始条件: G-PREP resolved before readiness; do not infer from source fixture
+終了条件: Every requested variant/checkpoint observed; no invented PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
       <c r="A12" s="27" t="inlineStr">
         <is>
           <t>対象外</t>
         </is>
       </c>
-      <c r="B12" s="10" t="n"/>
-    </row>
-    <row r="13" ht="32.1" customHeight="1">
+      <c r="B12" s="49" t="inlineStr">
+        <is>
+          <t>八義務の除外なし。実BLEND QAはsynthetic fixture対象外。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="61" customHeight="1">
       <c r="A13" s="27" t="inlineStr">
         <is>
           <t>制限事項</t>
         </is>
       </c>
-      <c r="B13" s="10" t="n"/>
-    </row>
-    <row r="14" ht="65.09999999999999" customHeight="1">
-      <c r="A14" s="27" t="inlineStr">
-        <is>
-          <t>ケース別の実行準備</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="n"/>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>G-PREP: concrete browser/request seams are not verified
+1件の未完了事項を対応するテストケースの準備に記載しています。
+5ケースの画面相対URLが未確認です。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="44" customHeight="1">
+      <c r="A14" s="27" t="inlineStr"/>
+      <c r="B14" s="49" t="inlineStr"/>
     </row>
     <row r="15" ht="32.1" customHeight="1">
       <c r="A15" s="30" t="inlineStr">
@@ -685,8 +910,8 @@
           <t>ケース数</t>
         </is>
       </c>
-      <c r="B16" s="32">
-        <f>COUNTA(A30:A30)</f>
+      <c r="B16" s="51">
+        <f>1</f>
         <v/>
       </c>
     </row>
@@ -696,118 +921,118 @@
           <t>バリエーション数</t>
         </is>
       </c>
-      <c r="B17" s="32">
-        <f>COUNTA(テスト!$A$5:$A$5)</f>
+      <c r="B17" s="51">
+        <f>2</f>
         <v/>
       </c>
     </row>
-    <row r="18" ht="32.1" customHeight="1">
-      <c r="A18" s="31" t="inlineStr">
-        <is>
-          <t>対象条件を満たす合格判定数</t>
-        </is>
-      </c>
-      <c r="B18" s="32">
-        <f>0</f>
+    <row r="18" ht="44" customHeight="1">
+      <c r="A18" s="49" t="inlineStr">
+        <is>
+          <t>対象条件を満たす合格ケース数</t>
+        </is>
+      </c>
+      <c r="B18" s="51">
+        <f>COUNTIF(C30:C30,"合格")</f>
         <v/>
       </c>
     </row>
-    <row r="19" ht="32.1" customHeight="1">
-      <c r="A19" s="31" t="inlineStr">
-        <is>
-          <t>対象条件を満たす不合格判定数</t>
-        </is>
-      </c>
-      <c r="B19" s="32">
-        <f>0</f>
+    <row r="19" ht="44" customHeight="1">
+      <c r="A19" s="49" t="inlineStr">
+        <is>
+          <t>対象条件を満たす不合格ケース数</t>
+        </is>
+      </c>
+      <c r="B19" s="51">
+        <f>COUNTIF(C30:C30,"不合格")</f>
         <v/>
       </c>
     </row>
-    <row r="20" ht="32.1" customHeight="1">
-      <c r="A20" s="31" t="inlineStr">
-        <is>
-          <t>実行不可数</t>
-        </is>
-      </c>
-      <c r="B20" s="32">
-        <f>0</f>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="49" t="inlineStr">
+        <is>
+          <t>実行不可バリエーション数</t>
+        </is>
+      </c>
+      <c r="B20" s="51">
+        <f>SUM('テストケース'!B90)</f>
         <v/>
       </c>
     </row>
-    <row r="21" ht="32.1" customHeight="1">
-      <c r="A21" s="31" t="inlineStr">
-        <is>
-          <t>実行省略数</t>
-        </is>
-      </c>
-      <c r="B21" s="32">
-        <f>0</f>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="49" t="inlineStr">
+        <is>
+          <t>実行省略バリエーション数</t>
+        </is>
+      </c>
+      <c r="B21" s="51">
+        <f>SUM('テストケース'!B91)</f>
         <v/>
       </c>
     </row>
-    <row r="22" ht="32.1" customHeight="1">
-      <c r="A22" s="31" t="inlineStr">
-        <is>
-          <t>未実行数</t>
-        </is>
-      </c>
-      <c r="B22" s="32">
-        <f>0</f>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="49" t="inlineStr">
+        <is>
+          <t>未実行バリエーション数</t>
+        </is>
+      </c>
+      <c r="B22" s="51">
+        <f>SUM('テストケース'!B92)</f>
         <v/>
       </c>
     </row>
-    <row r="23" ht="66" customHeight="1">
-      <c r="A23" s="31" t="inlineStr">
-        <is>
-          <t>対象条件を満たす合否判定数</t>
-        </is>
-      </c>
-      <c r="B23" s="32">
+    <row r="23" ht="44" customHeight="1">
+      <c r="A23" s="49" t="inlineStr">
+        <is>
+          <t>対象条件を満たす合否判定ケース数</t>
+        </is>
+      </c>
+      <c r="B23" s="51">
         <f>B18+B19</f>
         <v/>
       </c>
     </row>
-    <row r="24" ht="66" customHeight="1">
-      <c r="A24" s="31" t="inlineStr">
-        <is>
-          <t>合格数 / 対象条件を満たす合否判定数</t>
-        </is>
-      </c>
-      <c r="B24" s="33">
+    <row r="24" ht="44" customHeight="1">
+      <c r="A24" s="49" t="inlineStr">
+        <is>
+          <t>合格ケース数 / 対象条件を満たす合否判定ケース数</t>
+        </is>
+      </c>
+      <c r="B24" s="52">
         <f>IF(B23=0,"データなし",B18/B23)</f>
         <v/>
       </c>
     </row>
-    <row r="25" ht="66" customHeight="1">
-      <c r="A25" s="31" t="inlineStr">
-        <is>
-          <t>対象条件を満たす合否判定数 / 全バリエーション数</t>
-        </is>
-      </c>
-      <c r="B25" s="33">
-        <f>IF(B17=0,"データなし",B23/B17)</f>
+    <row r="25" ht="44" customHeight="1">
+      <c r="A25" s="49" t="inlineStr">
+        <is>
+          <t>対象条件を満たす合否判定ケース数 / 全ケース数</t>
+        </is>
+      </c>
+      <c r="B25" s="52">
+        <f>IF(B16=0,"データなし",B23/B16)</f>
         <v/>
       </c>
     </row>
-    <row r="26" ht="32.1" customHeight="1">
-      <c r="A26" s="31" t="inlineStr">
-        <is>
-          <t>合格未確認数</t>
-        </is>
-      </c>
-      <c r="B26" s="32">
-        <f>B17-B18</f>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="49" t="inlineStr">
+        <is>
+          <t>合格未確認ケース数</t>
+        </is>
+      </c>
+      <c r="B26" s="51">
+        <f>B16-B18</f>
         <v/>
       </c>
     </row>
-    <row r="27" ht="32.1" customHeight="1">
-      <c r="A27" s="31" t="inlineStr">
-        <is>
-          <t>無効な状態数</t>
-        </is>
-      </c>
-      <c r="B27" s="32">
-        <f>B17-SUM(0,0,0,0,0)</f>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="49" t="inlineStr">
+        <is>
+          <t>無効なバリエーション状態数</t>
+        </is>
+      </c>
+      <c r="B27" s="51">
+        <f>B17-SUM(B20:B22,SUM('テストケース'!B88),SUM('テストケース'!B89))</f>
         <v/>
       </c>
     </row>
@@ -832,11 +1057,8 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="32.1" customHeight="1">
-      <c r="A30" s="10" t="n"/>
-      <c r="B30" s="10" t="n"/>
-    </row>
   </sheetData>
+  <autoFilter ref="A29:C30"/>
   <mergeCells count="12">
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B6:C6"/>
@@ -851,7 +1073,9 @@
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B12:C12"/>
   </mergeCells>
+  <printOptions horizontalCentered="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -859,287 +1083,64 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0064748B"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <outlinePr summaryBelow="0" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="5"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="5"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="32.1" customHeight="1">
-      <c r="A1" s="37" t="inlineStr">
-        <is>
-          <t>テストケース配置例</t>
-        </is>
-      </c>
+      <c r="A1" s="70" t="inlineStr">
+        <is>
+          <t>テストケース詳細</t>
+        </is>
+      </c>
+      <c r="B1" s="71" t="n"/>
+      <c r="C1" s="71" t="n"/>
+      <c r="D1" s="71" t="n"/>
+      <c r="E1" s="71" t="n"/>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" s="38" t="inlineStr">
-        <is>
-          <t>以下は表示形式の例であり、実際のテストケースではありません。生成時に例を削除してソースの内容を書き込みます。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="12" customHeight="1"/>
+      <c r="A2" s="72" t="inlineStr"/>
+      <c r="B2" s="71" t="n"/>
+      <c r="C2" s="71" t="n"/>
+      <c r="D2" s="71" t="n"/>
+      <c r="E2" s="71" t="n"/>
+    </row>
+    <row r="3" ht="12" customHeight="1">
+      <c r="A3" s="71" t="n"/>
+      <c r="B3" s="71" t="n"/>
+      <c r="C3" s="71" t="n"/>
+      <c r="D3" s="71" t="n"/>
+      <c r="E3" s="71" t="n"/>
+    </row>
     <row r="4" ht="8" customHeight="1">
-      <c r="A4" s="13" t="n"/>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="39" t="inlineStr">
-        <is>
-          <t>[TC-ID] — [テストケース名]</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="n"/>
-      <c r="C5" s="16" t="n"/>
-      <c r="D5" s="16" t="n"/>
-      <c r="E5" s="16" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="40" t="inlineStr">
-        <is>
-          <t>状態</t>
-        </is>
-      </c>
-      <c r="B6" s="41" t="inlineStr">
-        <is>
-          <t>未実行</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="n"/>
-      <c r="D6" s="19" t="n"/>
-      <c r="E6" s="19" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="40" t="inlineStr">
-        <is>
-          <t>画面・機能</t>
-        </is>
-      </c>
-      <c r="B7" s="42" t="inlineStr">
-        <is>
-          <t>[画面・機能名]</t>
-        </is>
-      </c>
-      <c r="C7" s="19" t="n"/>
-      <c r="D7" s="40" t="inlineStr">
-        <is>
-          <t>相対URL</t>
-        </is>
-      </c>
-      <c r="E7" s="42" t="inlineStr">
-        <is>
-          <t>[/relative/path]</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="43" t="inlineStr">
-        <is>
-          <t>テスト条件</t>
-        </is>
-      </c>
-      <c r="B8" s="23" t="n"/>
-      <c r="C8" s="23" t="n"/>
-      <c r="D8" s="23" t="n"/>
-      <c r="E8" s="23" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="40" t="inlineStr">
-        <is>
-          <t>設定</t>
-        </is>
-      </c>
-      <c r="B9" s="42" t="inlineStr">
-        <is>
-          <t>• [初期条件・状態]</t>
-        </is>
-      </c>
-      <c r="C9" s="19" t="n"/>
-      <c r="D9" s="19" t="n"/>
-      <c r="E9" s="19" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="40" t="inlineStr">
-        <is>
-          <t>役割・権限</t>
-        </is>
-      </c>
-      <c r="B10" s="42" t="inlineStr">
-        <is>
-          <t>• [必要な役割・権限]</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="n"/>
-      <c r="D10" s="19" t="n"/>
-      <c r="E10" s="19" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="40" t="inlineStr">
-        <is>
-          <t>テストデータ</t>
-        </is>
-      </c>
-      <c r="B11" s="42" t="inlineStr">
-        <is>
-          <t>• [テストデータ・値]</t>
-        </is>
-      </c>
-      <c r="C11" s="19" t="n"/>
-      <c r="D11" s="19" t="n"/>
-      <c r="E11" s="19" t="n"/>
-    </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="43" t="inlineStr">
-        <is>
-          <t>操作</t>
-        </is>
-      </c>
-      <c r="B12" s="23" t="n"/>
-      <c r="C12" s="23" t="n"/>
-      <c r="D12" s="23" t="n"/>
-      <c r="E12" s="23" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="40" t="inlineStr">
-        <is>
-          <t>ステップ 1</t>
-        </is>
-      </c>
-      <c r="B13" s="42" t="inlineStr">
-        <is>
-          <t>[最初の操作]</t>
-        </is>
-      </c>
-      <c r="C13" s="19" t="n"/>
-      <c r="D13" s="19" t="n"/>
-      <c r="E13" s="19" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="40" t="inlineStr">
-        <is>
-          <t>ステップ 2</t>
-        </is>
-      </c>
-      <c r="B14" s="42" t="inlineStr">
-        <is>
-          <t>[次の操作]</t>
-        </is>
-      </c>
-      <c r="C14" s="19" t="n"/>
-      <c r="D14" s="19" t="n"/>
-      <c r="E14" s="19" t="n"/>
-    </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="43" t="inlineStr">
-        <is>
-          <t>期待結果</t>
-        </is>
-      </c>
-      <c r="B15" s="23" t="n"/>
-      <c r="C15" s="23" t="n"/>
-      <c r="D15" s="23" t="n"/>
-      <c r="E15" s="23" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="40" t="inlineStr">
-        <is>
-          <t>1.</t>
-        </is>
-      </c>
-      <c r="B16" s="42" t="inlineStr">
-        <is>
-          <t>[比較可能な期待結果]</t>
-        </is>
-      </c>
-      <c r="C16" s="19" t="n"/>
-      <c r="D16" s="19" t="n"/>
-      <c r="E16" s="19" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="40" t="inlineStr">
-        <is>
-          <t>2.</t>
-        </is>
-      </c>
-      <c r="B17" s="42" t="inlineStr">
-        <is>
-          <t>[維持すべき動作・データ]</t>
-        </is>
-      </c>
-      <c r="C17" s="19" t="n"/>
-      <c r="D17" s="19" t="n"/>
-      <c r="E17" s="19" t="n"/>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="43" t="inlineStr">
-        <is>
-          <t>実際の結果</t>
-        </is>
-      </c>
-      <c r="B18" s="23" t="n"/>
-      <c r="C18" s="23" t="n"/>
-      <c r="D18" s="23" t="n"/>
-      <c r="E18" s="23" t="n"/>
-    </row>
-    <row r="19" ht="64" customHeight="1">
-      <c r="A19" s="36" t="n"/>
-      <c r="B19" s="19" t="n"/>
-      <c r="C19" s="19" t="n"/>
-      <c r="D19" s="19" t="n"/>
-      <c r="E19" s="19" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="40" t="inlineStr">
-        <is>
-          <t>証拠画像</t>
-        </is>
-      </c>
-      <c r="B20" s="19" t="n"/>
-      <c r="C20" s="19" t="n"/>
-      <c r="D20" s="19" t="n"/>
-      <c r="E20" s="19" t="n"/>
-    </row>
-    <row r="21" ht="90" customHeight="1">
-      <c r="A21" s="36" t="n"/>
-      <c r="B21" s="19" t="n"/>
-      <c r="C21" s="19" t="n"/>
-      <c r="D21" s="19" t="n"/>
-      <c r="E21" s="19" t="n"/>
+      <c r="A4" s="73" t="n"/>
+      <c r="B4" s="71" t="n"/>
+      <c r="C4" s="71" t="n"/>
+      <c r="D4" s="71" t="n"/>
+      <c r="E4" s="71" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="B7:C7"/>
+  <mergeCells count="1">
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="B14:E14"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="A18:E18"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E15 E16" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
       <formula1>"合格,不合格,実行不可,実行省略,未実行"</formula1>
     </dataValidation>
   </dataValidations>
+  <printOptions horizontalCentered="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>